<commit_message>
Embed per-name returns verdicts + add status/priorities recalibration
Audit workbook Sheet 2 now records, for each of the 7 absent constituents,
the current SEC entity, corporate-action date, membership snapshots, and a
USE/DROP/truncate decision grounded in rename-date vs membership-window
analysis (SNSE/ELOXD/BHM = use; MNMD/GMGI/RENB/QVCGB = drop/truncate).
Adds a status-and-priorities memo: contract phase complete, critical path is
ground-truth set -> pilot extraction engine -> scale -> metrics -> analytics.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VyNEAGV7EoeTqwGq3GSDXN
</commit_message>
<xml_diff>
--- a/Morningstar_Returns_Coverage_Audit.xlsx
+++ b/Morningstar_Returns_Coverage_Audit.xlsx
@@ -2261,14 +2261,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2295,17 +2295,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>cik_map_name</t>
+          <t>current_sec_entity</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>isin</t>
+          <t>corporate_action</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>cusip</t>
+          <t>membership_snapshots</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -2315,12 +2315,12 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>years_in_index</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>retrieval_guidance</t>
+          <t>guidance</t>
         </is>
       </c>
     </row>
@@ -2347,28 +2347,26 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Aruba Networks Inc</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>US0431761065</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>043176106</t>
+          <t>4.30.15</t>
         </is>
       </c>
       <c r="H2" t="n">
         <v>0.2909</v>
       </c>
-      <c r="I2" t="n">
-        <v>1</v>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2395,28 +2393,26 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Swift Transportation Co</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>US87074U1016</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>87074U101</t>
+          <t>4.30.15,4.30.16,4.30.17</t>
         </is>
       </c>
       <c r="H3" t="n">
         <v>0.2278</v>
       </c>
-      <c r="I3" t="n">
-        <v>3</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2443,28 +2439,26 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Auspex Pharmaceuticals Inc</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>US05211J1025</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>05211J102</t>
+          <t>4.30.15</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>0.1162</v>
       </c>
-      <c r="I4" t="n">
-        <v>1</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2491,28 +2485,26 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>South Jersey Industries Inc</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>US8385181081</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>838518108</t>
+          <t>4.30.19,4.30.20,4.30.21</t>
         </is>
       </c>
       <c r="H5" t="n">
         <v>0.1046</v>
       </c>
-      <c r="I5" t="n">
-        <v>3</v>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2539,28 +2531,26 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Kofax Ltd</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>BMG5307C1055</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>G5307C105</t>
+          <t>4.30.15</t>
         </is>
       </c>
       <c r="H6" t="n">
         <v>0.0906</v>
       </c>
-      <c r="I6" t="n">
-        <v>1</v>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2587,28 +2577,26 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Hyperion Therapeutics Inc</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>US44915N1019</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>44915N101</t>
+          <t>4.30.15</t>
         </is>
       </c>
       <c r="H7" t="n">
         <v>0.0551</v>
       </c>
-      <c r="I7" t="n">
-        <v>1</v>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2635,28 +2623,26 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Horizon Global Corp</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>US44052W1045</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>44052W104</t>
+          <t>4.30.16,4.30.17,4.30.18</t>
         </is>
       </c>
       <c r="H8" t="n">
         <v>0.0328</v>
       </c>
-      <c r="I8" t="n">
-        <v>3</v>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2683,28 +2669,26 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>First Tracks Biotherapeutics Inc</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>US3371851029</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>337185102</t>
+          <t>4.30.26</t>
         </is>
       </c>
       <c r="H9" t="n">
         <v>0.025</v>
       </c>
-      <c r="I9" t="n">
-        <v>1</v>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2731,28 +2715,26 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Norcraft Companies Inc</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>US65557Y1055</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>65557Y105</t>
+          <t>4.30.15</t>
         </is>
       </c>
       <c r="H10" t="n">
         <v>0.0213</v>
       </c>
-      <c r="I10" t="n">
-        <v>1</v>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2779,28 +2761,26 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cellular Dynamics International Inc</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>US15117V1098</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>15117V109</t>
+          <t>4.30.15</t>
         </is>
       </c>
       <c r="H11" t="n">
         <v>0.0167</v>
       </c>
-      <c r="I11" t="n">
-        <v>1</v>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2827,28 +2807,26 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Entropic Communications Inc</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>US29384R1059</t>
-        </is>
-      </c>
+          <t>(acquired/delisted)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>29384R105</t>
+          <t>4.30.15</t>
         </is>
       </c>
       <c r="H12" t="n">
         <v>0.002</v>
       </c>
-      <c r="I12" t="n">
-        <v>1</v>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>BACKFILL or DROP</t>
+        </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Series dropped at delisting/acquisition. Retrieve from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify entity name+dates match.</t>
+          <t>Series dropped at delisting/acquisition. Backfill from Bloomberg/FactSet/CRSP by CUSIP/ISIN for the MEMBERSHIP window only; verify name+dates. Else drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -2875,28 +2853,30 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Mind Medicine Inc Ordinary Shares</t>
+          <t>Definium Therapeutics (DFTX)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>CA60255C8850</t>
+          <t>2026-01-12 rename</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>60255C885</t>
+          <t>4.30.25</t>
         </is>
       </c>
       <c r="H13" t="n">
         <v>0.0393</v>
       </c>
-      <c r="I13" t="n">
-        <v>1</v>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>DROP (or truncate @2026-01-12)</t>
+        </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Holdings CUSIP/ISIN is STALE (reorg/redomicile/rename). Search Morningstar by CIK or current ticker; VERIFY returned entity = expected name during membership months. Reject any CUSIP that resolves to a different company (recycled).</t>
+          <t>In index 4.30.25; rename falls INSIDE membership window. 0.039% wt -&gt; drop w/ disclosure, or truncate returns at rename.</t>
         </is>
       </c>
     </row>
@@ -2923,28 +2903,30 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Eloxx Pharmaceuticals Inc</t>
+          <t>Eloxx Pharmaceuticals (ELOX/ELOXD)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>US29014R1032</t>
+          <t>none</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>29014R103</t>
+          <t>4.30.19,4.30.20,4.30.21</t>
         </is>
       </c>
       <c r="H14" t="n">
         <v>0.0247</v>
       </c>
-      <c r="I14" t="n">
-        <v>3</v>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Holdings CUSIP/ISIN is STALE (reorg/redomicile/rename). Search Morningstar by CIK or current ticker; VERIFY returned entity = expected name during membership months. Reject any CUSIP that resolves to a different company (recycled).</t>
+          <t>Same entity; identifier-match miss. Pull by current ticker ELOX (likely already in file).</t>
         </is>
       </c>
     </row>
@@ -2971,28 +2953,30 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sensei Biotherapeutics Inc Ordinary Shares</t>
+          <t>Faeth Therapeutics (SNSE)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>US81728A1088</t>
+          <t>2026-06-16 rename</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>81728A108</t>
+          <t>4.30.21</t>
         </is>
       </c>
       <c r="H15" t="n">
         <v>0.0057</v>
       </c>
-      <c r="I15" t="n">
-        <v>1</v>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>USE (window only)</t>
+        </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Holdings CUSIP/ISIN is STALE (reorg/redomicile/rename). Search Morningstar by CIK or current ticker; VERIFY returned entity = expected name during membership months. Reject any CUSIP that resolves to a different company (recycled).</t>
+          <t>In index 4.30.21; rename 5yr later. Pull series, keep ONLY 2021-22 membership months; confirm history continuous.</t>
         </is>
       </c>
     </row>
@@ -3019,28 +3003,30 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Golden Matrix Group Inc</t>
+          <t>Meridian Holdings (MRDN)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>US3810983003</t>
+          <t>2026-03-03 rename</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>381098300</t>
+          <t>4.30.25</t>
         </is>
       </c>
       <c r="H16" t="n">
         <v>0.0034</v>
       </c>
-      <c r="I16" t="n">
-        <v>1</v>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>DROP</t>
+        </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Holdings CUSIP/ISIN is STALE (reorg/redomicile/rename). Search Morningstar by CIK or current ticker; VERIFY returned entity = expected name during membership months. Reject any CUSIP that resolves to a different company (recycled).</t>
+          <t>In index 4.30.25; rename inside window. 0.003% wt -&gt; drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -3067,28 +3053,30 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bluerock Homes Trust Inc Ordinary Shares - Class A</t>
+          <t>Bluerock Homes Trust (BHM, NYSE)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>US09631H1005</t>
+          <t>none</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>09631H100</t>
+          <t>4.30.23</t>
         </is>
       </c>
       <c r="H17" t="n">
         <v>0.0023</v>
       </c>
-      <c r="I17" t="n">
-        <v>1</v>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>USE</t>
+        </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Holdings CUSIP/ISIN is STALE (reorg/redomicile/rename). Search Morningstar by CIK or current ticker; VERIFY returned entity = expected name during membership months. Reject any CUSIP that resolves to a different company (recycled).</t>
+          <t>Same entity; identifier-match miss. Pull directly by ticker BHM.</t>
         </is>
       </c>
     </row>
@@ -3115,28 +3103,30 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Renovaro Inc</t>
+          <t>Lunai Bioworks (LNAI)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>US29350E1047</t>
+          <t>2025-08-26 rename</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>29350E104</t>
+          <t>4.30.20,4.30.25</t>
         </is>
       </c>
       <c r="H18" t="n">
         <v>0.0022</v>
       </c>
-      <c r="I18" t="n">
-        <v>2</v>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>DROP</t>
+        </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Holdings CUSIP/ISIN is STALE (reorg/redomicile/rename). Search Morningstar by CIK or current ticker; VERIFY returned entity = expected name during membership months. Reject any CUSIP that resolves to a different company (recycled).</t>
+          <t>In index 4.30.25; rename right after snapshot, window mostly successor. 0.002% wt -&gt; drop w/ disclosure.</t>
         </is>
       </c>
     </row>
@@ -3163,28 +3153,30 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>QVC Group Inc Ordinary Shares - Series B</t>
+          <t>QVC Inc (QVCCQ, OTC/distressed)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>US74915M2098</t>
+          <t>distressed/OTC</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>74915M209</t>
+          <t>4.30.24,4.30.25</t>
         </is>
       </c>
       <c r="H19" t="n">
         <v>0.0005</v>
       </c>
-      <c r="I19" t="n">
-        <v>2</v>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>DROP</t>
+        </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Holdings CUSIP/ISIN is STALE (reorg/redomicile/rename). Search Morningstar by CIK or current ticker; VERIFY returned entity = expected name during membership months. Reject any CUSIP that resolves to a different company (recycled).</t>
+          <t>0.0005% wt; now bankrupt OTC. Drop w/ disclosure.</t>
         </is>
       </c>
     </row>

</xml_diff>